<commit_message>
Repositorio propio: fuera todo lo que amarraba al curso
Es un proyecto personal, no material institucional, así que no debe remitir
a ninguna universidad ni suponer que el lector está matriculado.

- La plantilla decía «renombre el archivo: S1-Ideas-Apellido-Nombre.xlsx»
  (nomenclatura de entrega de un curso) y proponía buscar molestias en «su
  universidad» y «el trabajo de sus papás», que asumen estudiante joven.
  Generalizado. Verificado que las fórmulas y las listas desplegables
  sobrevivieron a la edición.
- El README hablaba de «los cinco sectores del curso».
- LICENSE: sale la nota provisional sobre propiedad intelectual, entra la
  autoría.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descubrir/01-generador-de-ideas/plantilla-ideas.xlsx
+++ b/descubrir/01-generador-de-ideas/plantilla-ideas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Molestias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SCAMPER" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Molestias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCAMPER" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -112,11 +112,84 @@
         <color rgb="009FE5E2"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="009FE5E2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="009FE5E2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009FE5E2"/>
+      </right>
+      <top style="thin">
+        <color rgb="009FE5E2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009FE5E2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="009FE5E2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="009FE5E2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009FE5E2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="009FE5E2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009FE5E2"/>
+      </right>
+      <top style="thin">
+        <color rgb="009FE5E2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009FE5E2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -153,6 +226,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -620,7 +699,7 @@
         <f>IF(COUNTA(B2:B300)&gt;=30,"Ya pasó el mínimo de 30","Le faltan "&amp;(30-COUNTA(B2:B300))&amp;" para el mínimo de 30")</f>
         <v/>
       </c>
-      <c r="G5" s="10" t="n"/>
+      <c r="G5" s="14" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -646,10 +725,10 @@
 • Las ideas de SCAMPER van en las dos hojas: acá con Origen = S, y en la hoja SCAMPER junto a su letra.
 • No borre nada. Las ideas obvias, repetidas y malas también se entregan: son la prueba de que generó sin frenar.
 • Si pasa de 34, agregue filas y siga numerando.
-• Antes de subirlo, renombre el archivo: S1-Ideas-Apellido-Nombre.xlsx</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="n"/>
+• Guarde el archivo con su nombre antes de compartirlo.</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -658,8 +737,8 @@
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -668,8 +747,8 @@
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -678,8 +757,8 @@
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="4" t="n">
@@ -688,8 +767,8 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -698,8 +777,8 @@
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -708,8 +787,8 @@
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -718,8 +797,8 @@
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -728,8 +807,8 @@
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="4" t="n">
@@ -738,8 +817,8 @@
       <c r="B16" s="5" t="n"/>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -748,8 +827,8 @@
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="17" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -758,8 +837,8 @@
       <c r="B18" s="5" t="n"/>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -768,8 +847,8 @@
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="17" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -778,8 +857,8 @@
       <c r="B20" s="5" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="19" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="n">
@@ -972,90 +1051,90 @@
 Cosas que lo sacan de casillas, le hacen perder tiempo, le cuestan plata o le dan pereza. A usted, a su familia, a sus compañeros, o a alguien que vio esta semana.
 No piense en negocios todavía. Solo molestias.
 Sirve mirar en estos frentes:
-· su universidad
+· su estudio o su trabajo
 · su casa
 · su transporte
 · su plata
 · su salud
 · su barrio
-· el trabajo de sus papás
+· el oficio de alguien cercano
 · algo que vio en la calle y le pareció absurdo
 Esta hoja se entrega. Es la evidencia de que arrancó por el problema y no por la solución.</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
+      <c r="D4" s="15" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="5" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="17" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="5" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="17" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="5" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="17" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="5" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
+      <c r="C8" s="16" t="n"/>
+      <c r="D8" s="17" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="5" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="17" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="5" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="17" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="5" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="17" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="5" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="17" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="5" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="17" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="5" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="17" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="5" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="17" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="5" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="17" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="17" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1139,7 +1218,7 @@
           <t>Qué pregunta cada letra</t>
         </is>
       </c>
-      <c r="E4" s="10" t="n"/>
+      <c r="E4" s="14" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
@@ -1169,7 +1248,7 @@
 No se salte una letra porque «no aplica». Que no aplique es justo el momento en que la técnica lo obliga a pensar distinto: escriba algo aunque sea malo.</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n"/>
+      <c r="E5" s="15" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -1178,8 +1257,8 @@
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="17" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
@@ -1188,8 +1267,8 @@
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="17" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
@@ -1198,8 +1277,8 @@
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="17" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -1208,8 +1287,8 @@
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
@@ -1218,8 +1297,8 @@
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="17" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
@@ -1228,8 +1307,8 @@
         </is>
       </c>
       <c r="B11" s="5" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="17" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
@@ -1238,8 +1317,8 @@
         </is>
       </c>
       <c r="B12" s="5" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="17" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -1248,8 +1327,8 @@
         </is>
       </c>
       <c r="B13" s="5" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="17" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
@@ -1258,8 +1337,8 @@
         </is>
       </c>
       <c r="B14" s="5" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="17" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
@@ -1268,86 +1347,86 @@
         </is>
       </c>
       <c r="B15" s="5" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="17" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="5" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="17" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="5" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="17" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="5" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="17" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="5" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="17" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="5" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="17" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="5" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="17" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="5" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="17" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="5" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="17" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="5" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="17" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="5" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="17" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="5" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="17" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="5" t="n"/>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="10" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="17" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="5" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="19" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="6" t="n"/>

</xml_diff>